<commit_message>
Move initial reader positions to Excel files, remove hardcoded defaults
- LecteurDB.py / SP_LecteurDB.py: removed all DEFAULT_LECTEURS constants.
  _ensure_file() now only creates an empty file (headers only) if missing.
  Single source of truth is the Excel file in Parametres/.

- Parametres/lecteurs.xlsx: Lane 5000 + Move 5000 initial positions.
- Parametres/sp_lecteurs.xlsx: iPhone SE, iPhone 13, Samsung A34,
  Samsung S23, Samsung A15, Redmi 13C initial positions.

https://claude.ai/code/session_012Qyz7eWCpt1RXWrua4sBWk
</commit_message>
<xml_diff>
--- a/Parametres/lecteurs.xlsx
+++ b/Parametres/lecteurs.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,32 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="000054A4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8F0FB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -65,13 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -437,283 +413,105 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Nom</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>y</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>z</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>rX</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>rY</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>rZ</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>topZ</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Lane 5000</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" t="n">
         <v>-0.4547756256699072</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" t="n">
         <v>0.09449841328596138</v>
       </c>
-      <c r="D2" s="2" t="n">
-        <v>0.180246450696463</v>
-      </c>
-      <c r="E2" s="2" t="n">
+      <c r="D2" t="n">
+        <v>0.2104684407509641</v>
+      </c>
+      <c r="E2" t="n">
         <v>-2.216230493253284</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" t="n">
         <v>2.225071346999853</v>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="G2" t="n">
         <v>0.01629001438342314</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H2" t="n">
         <v>0.399821937815115</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Move 5000</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" t="n">
         <v>-0.4540141593144729</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" t="n">
         <v>0.03158068214332013</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" t="n">
         <v>0.3087100442018794</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E3" t="n">
         <v>-2.20372181601157</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="F3" t="n">
         <v>2.237287604332674</v>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="G3" t="n">
         <v>0.01616534026994103</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="H3" t="n">
         <v>0.5025886995214306</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>iPhone SE</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>-0.4535050711611319</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>0.09746050997975206</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>0.1628971910211756</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>-2.231798624387687</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>2.208553388261561</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>0.01263574497103918</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>0.399821937815115</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>iPhone 13</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>-0.4530451975084202</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>0.09109465497697321</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>0.1623321775801928</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>-2.231812791929215</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>2.20836277121875</v>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>0.01254847786091072</v>
-      </c>
-      <c r="H5" s="3" t="n">
-        <v>0.399821937815115</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Samsung A34</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>-0.437542675153976</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>0.05571605275012892</v>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>0.1632553872558145</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>-2.228789920172243</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>2.211582666496985</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>0.01273950301260789</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>0.399821937815115</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Samsung S23</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>-0.4421296622829857</v>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>0.00187198604837873</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>0.1640113525916818</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>-2.21201284730284</v>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>2.228231632546852</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>0.0127072456801193</v>
-      </c>
-      <c r="H7" s="3" t="n">
-        <v>0.399821937815115</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Samsung A15</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>-0.4386549445573203</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>0.0774494613480611</v>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>0.166747999898712</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>-2.216200668681918</v>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>2.22500596381785</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>0.01613230061897039</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>0.399821937815115</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Redmi 13C</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>-0.4342770051859024</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>0.07549404718371988</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>0.1650135223170027</v>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>2.208902454165429</v>
-      </c>
-      <c r="F9" s="3" t="n">
-        <v>-2.227313501553085</v>
-      </c>
-      <c r="G9" s="3" t="n">
-        <v>0.002980852769627379</v>
-      </c>
-      <c r="H9" s="3" t="n">
-        <v>0.399821937815115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>